<commit_message>
-se continuo con el analisis de las metricas realizadas en el 1C 2026 en Programacion Concurrente
</commit_message>
<xml_diff>
--- a/metricas_realizadas/Prog-Concurrente/Analisis de metricas/Metricas utilizadas 1C 2026.xlsx
+++ b/metricas_realizadas/Prog-Concurrente/Analisis de metricas/Metricas utilizadas 1C 2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\proyecto_code_ia\metricas_realizadas\Prog-Concurrente\Analisis de metricas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA0F5ABF-7B43-4CC8-B34F-A2BBC327DA0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC4DDF69-97E7-44D9-96B0-6F4641104620}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Resumen del trabajo" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="125">
   <si>
     <t>Grupo</t>
   </si>
@@ -175,13 +175,6 @@
     <t>Rubrica</t>
   </si>
   <si>
-    <t xml:space="preserve">sincronización OK
-deadlocks OK
-race condition OK
-exclusión mutua OK
-</t>
-  </si>
-  <si>
     <t>medicion</t>
   </si>
   <si>
@@ -259,14 +252,6 @@
 uso de memoria promedio = 68 MB</t>
   </si>
   <si>
-    <t xml:space="preserve">hubo que hacer varios refinamientos porque habia problemas de concurrencia
-sincronización OK
-deadlocks OK
-race condition OK
-exclusión mutua OK
-</t>
-  </si>
-  <si>
     <t>Haiku 4.5
 Opus 4.7</t>
   </si>
@@ -361,35 +346,6 @@
   </si>
   <si>
     <t>SpotBugs y analisis estatico</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <u/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>usando Opus en los dos etapas:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-sincronización OK
-deadlocks OK
-race condition OK
-exclusión mutua OK
-</t>
-    </r>
   </si>
   <si>
     <r>
@@ -550,23 +506,1156 @@
 </t>
   </si>
   <si>
+    <t>IDE sin especificar</t>
+  </si>
+  <si>
+    <t>sistema simulado de delivery de pedido ya</t>
+  </si>
+  <si>
+    <t>La CC mide el número de caminos lógicamente independientes (ramificaciones). A mayor CC, más casos de prueba y más riesgo de defectos</t>
+  </si>
+  <si>
+    <t>utiliza la metrica de Halstead
+MI=171−5.2ln(V)−0.23(CC)−16.2ln(LOC)</t>
+  </si>
+  <si>
+    <t>MI más bajo, indicando menor facilidad de mantenimiento. En cambio, valores altos de MI indican código más simple, legible y fácil de modificar.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sincronización Alta
+deadlocks Alta
+race condition Alta
+exclusión mutua Alta
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hubo que hacer varios refinamientos porque habia problemas de concurrencia
+sincronización Media
+deadlocks Alta
+race condition Alta
+exclusión mutua Alta
+</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>usando Opus en los dos etapas:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+sincronización Alta
+deadlocks Alta
+race condition Alta
+exclusión mutua Alta
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>CC con Gemini</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+CC promedio total = 2,10.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">CC con Claude Sonnet
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>CC promedio total = 2,42.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>MI con Gemini:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">= 55 de 100
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>MI con Claude Sonnet</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>:= 39,82 de 100</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Con Gemini =</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">12 Threads en simultaneo
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Con Claude Sonnet</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> =  12 Threads en simultaneo</t>
+    </r>
+  </si>
+  <si>
+    <t>usando psutil</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Con Gemini =
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Uso CPU promedio=0.5%
+Uso memoria promedio= 20 mb
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Con Claude Sonnet =</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Uso CPU promedio=0.2%
+Uso memoria promedio= 15 mb</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Con Gemimi=</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">2800 tokens
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Con Claude Sonnet = </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>7418 tokens</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve"> 1 refinamientos</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Con Gemini =</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+sincronización Media
+deadlocks Alta
+race condition Alta
+exclusión mutua Alta
+startvation = Alta
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Con Claude Sonnet =
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>sincronización Media
+deadlocks Alta
+race condition Alta
+exclusión mutua Alta
+startvation = media (al emplear cola sin prioridades)</t>
+    </r>
+  </si>
+  <si>
+    <t>0 refinamientos</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>CC con Gemini</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+CC promedio total = 2,10.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">CC con Claude Sonnet
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">CC promedio total = 2,42.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+CC con GPT
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">CC promedio total = 3,9.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+CC con Deepseek:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>CC promedio total = 3,5.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>MI con Gemini:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">= 55 de 100
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>MI con Claude Sonnet</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">:= 39,82 de 100
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>MI con GPT :=</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 46,86 de 100
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>MI con Deepseek :=</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 31,82 de 100</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Con Gemini =</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">12 Threads en simultaneo
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Con Claude Sonnet</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> =  12 Threads en simultaneo</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Con GPT =  </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">12 Threads en simultaneo
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Con Deepseek =</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">  12 Threads en simultaneo</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Con Gemini =
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Uso CPU promedio=0.5%
+Uso memoria promedio= 20 mb
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Con Claude Sonnet =</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Uso CPU promedio=0.2%
+Uso memoria promedio= 15 mb
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Con GPT =</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Uso CPU promedio=10,61%
+Uso memoria promedio= 20 mb
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Con Deepseek=</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Uso CPU promedio=12,43%
+Uso memoria promedio= 20 mb</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Con Gemimi=</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">2800 tokens
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Con Claude Sonnet = </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">7418 tokens
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Con GPT </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">= 5955 tokens
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Con Deepseek =</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 6670</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> tokens</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Con Gemini =</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+sincronización Media
+deadlocks Alta
+race condition Alta
+exclusión mutua Alta
+startvation = Alta
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Con Claude Sonnet =
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">sincronización Media
+deadlocks Alta
+race condition Alta
+exclusión mutua Alta
+startvation = media (al emplear cola sin prioridades)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Con GPT Mini =</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+sincronización Media
+deadlocks Media
+race condition Media
+exclusión mutua Media
+startvation = media
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Con Deepseek =</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+sincronización Media
+deadlocks Media
+race condition Media
+exclusión mutua Media
+startvation = media</t>
+    </r>
+  </si>
+  <si>
+    <t>video juego 2D Sheriff</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Claude Sonnet 4
+Claude Opus 4
+</t>
+  </si>
+  <si>
     <t>Gemini 3.1 pro
-Cloude Sonnet 4.6
+Claude Sonnet 4.6
 GPT 5  Mini
 Deepsek v4 Mini Flash</t>
   </si>
   <si>
-    <t>IDE sin especificar</t>
-  </si>
-  <si>
-    <t>sistema simulado de delivery de pedido ya</t>
+    <t xml:space="preserve">prompting tecnico </t>
+  </si>
+  <si>
+    <t>prompt inicial basico y refinamientos dividio por bloques tematicos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">aproximadamente 80 refinamientos </t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">utiliza la metrica de Halstead
+MI=171−5.2ln(V)−0.23(CC)−16.2ln(LOC)
+detección de good smells usando Fowler y heuristica de Riel
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>utiliza script propio para calculo de MI acorde a los resultados de lizard</t>
+    </r>
+  </si>
+  <si>
+    <t>utiliza herramienta jcmd Thread.print. Toma 3 snapshot en diferentes momentos</t>
+  </si>
+  <si>
+    <t>usa ps (CPU%/RSS) + jcmd GC.heap_info.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">aproximadamente 750000 Tokens </t>
+  </si>
+  <si>
+    <t xml:space="preserve">CC promedio total = 2.3,cant de funciones total=913 (excelente)
+CC función más compleja =44 
+porcentaje de funciones con cc&gt;10=2,2% </t>
+  </si>
+  <si>
+    <t xml:space="preserve">MI promedio=41.7 (Bueno)
+MI Minimo =4.3(inmantenible)(Archivo Game.java)
+</t>
+  </si>
+  <si>
+    <t>1 solo hilo activo todo el tiempo del propio juego (Correcto)
+36 hilos del sistema de VM de java+GC+ audio+ Swing AWT</t>
+  </si>
+  <si>
+    <t>sincronización Alta
+deadlocks Alta
+race condition Alta
+exclusión mutua Alta
+startvation = Alta
+(Excelente)</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">tiene en cuenta todo los multiples cores y el uso del sistema VM de java y demás. Por eso da muy grande los valores:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>uso CPU promedio=203,33%  (Aceptable)
+uso de memoria promedio=200MB  (Aceptable)</t>
+    </r>
+  </si>
+  <si>
+    <t>Claude Opus 7</t>
+  </si>
+  <si>
+    <t>Python</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Procesamiento concurrente de imaganes </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Utilizaron la herramienta Radon para Python
+ CC = E – N + 2P. 
+Utiliza clasificación de McCabe
+</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Utilizaron la herramienta Lizard para java</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+ CC = E – N + 2P. 
+Utiliza clasificación de McCabe
+</t>
+    </r>
+  </si>
+  <si>
+    <t>CC promedio=3</t>
+  </si>
+  <si>
+    <t>utiliza la metrica de Halstead con Radon
+MI=171−5.2ln(V)−0.23(CC)−16.2ln(LOC)</t>
+  </si>
+  <si>
+    <t>Radon normaliza el MI resultante dando que todos los módulos tienen buena buena capacidad de mantenimiento
+ya que el valor de indice mas chico  es igual a 74</t>
+  </si>
+  <si>
+    <t xml:space="preserve">en las pruebas se usan 6 threads. 
+</t>
+  </si>
+  <si>
+    <t>Uso promedio CPU = 304%
+uso promedio memoria=396mb</t>
+  </si>
+  <si>
+    <t>2216 tokens</t>
+  </si>
+  <si>
+    <t>sincronización Alta
+deadlocks media
+race condition Alta
+exclusión mutua Alta
+startvation = Alta</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -602,6 +1691,21 @@
       <u/>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -719,7 +1823,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -800,6 +1904,18 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1176,7 +2292,7 @@
         <v>9</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="101.5" x14ac:dyDescent="0.35">
@@ -1199,7 +2315,7 @@
         <v>26</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="101.5" x14ac:dyDescent="0.35">
@@ -1207,22 +2323,22 @@
         <v>3</v>
       </c>
       <c r="B3" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="D3" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="E3" s="6" t="s">
         <v>50</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>51</v>
       </c>
       <c r="F3" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="101.5" x14ac:dyDescent="0.35">
@@ -1230,13 +2346,13 @@
         <v>4</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E4" s="8" t="s">
         <v>11</v>
@@ -1245,7 +2361,7 @@
         <v>26</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="H4" s="3"/>
     </row>
@@ -1254,32 +2370,68 @@
         <v>5</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>78</v>
+        <v>100</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="F5" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B6" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>7</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>101</v>
       </c>
     </row>
   </sheetData>
@@ -1292,11 +2444,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{485790A4-37CE-4FFB-B88A-82F970BB1079}">
-  <dimension ref="A1:E37"/>
+  <sheetPr codeName="Hoja1"/>
+  <dimension ref="A1:E64"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="30.26953125" customWidth="1"/>
-    <col min="3" max="3" width="32.36328125" customWidth="1"/>
+    <col min="3" max="3" width="37.90625" customWidth="1"/>
     <col min="4" max="4" width="50" customWidth="1"/>
     <col min="5" max="5" width="26" customWidth="1"/>
   </cols>
@@ -1359,7 +2512,7 @@
         <v>24</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E4" s="19"/>
     </row>
@@ -1411,7 +2564,7 @@
         <v>41</v>
       </c>
       <c r="D8" s="21" t="s">
-        <v>42</v>
+        <v>80</v>
       </c>
       <c r="E8" s="19"/>
     </row>
@@ -1421,20 +2574,20 @@
         <v>21</v>
       </c>
       <c r="C9" s="21" t="s">
+        <v>42</v>
+      </c>
+      <c r="D9" s="20" t="s">
         <v>43</v>
-      </c>
-      <c r="D9" s="20" t="s">
-        <v>44</v>
       </c>
       <c r="E9" s="19"/>
     </row>
     <row r="10" spans="1:5" ht="58" x14ac:dyDescent="0.35">
       <c r="A10" s="32"/>
       <c r="B10" s="22" t="s">
+        <v>45</v>
+      </c>
+      <c r="C10" s="23" t="s">
         <v>46</v>
-      </c>
-      <c r="C10" s="23" t="s">
-        <v>47</v>
       </c>
       <c r="D10" s="24"/>
       <c r="E10" s="25"/>
@@ -1447,10 +2600,10 @@
         <v>16</v>
       </c>
       <c r="C11" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="D11" s="11" t="s">
         <v>52</v>
-      </c>
-      <c r="D11" s="11" t="s">
-        <v>53</v>
       </c>
       <c r="E11" s="13"/>
     </row>
@@ -1460,10 +2613,10 @@
         <v>17</v>
       </c>
       <c r="C12" s="28" t="s">
+        <v>53</v>
+      </c>
+      <c r="D12" s="16" t="s">
         <v>54</v>
-      </c>
-      <c r="D12" s="16" t="s">
-        <v>55</v>
       </c>
       <c r="E12" s="18"/>
     </row>
@@ -1473,10 +2626,10 @@
         <v>18</v>
       </c>
       <c r="C13" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="D13" s="16" t="s">
         <v>56</v>
-      </c>
-      <c r="D13" s="16" t="s">
-        <v>57</v>
       </c>
       <c r="E13" s="19"/>
     </row>
@@ -1487,7 +2640,7 @@
       </c>
       <c r="C14" s="16"/>
       <c r="D14" s="16" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E14" s="19"/>
     </row>
@@ -1497,10 +2650,10 @@
         <v>19</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D15" s="26" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E15" s="19"/>
     </row>
@@ -1510,10 +2663,10 @@
         <v>20</v>
       </c>
       <c r="C16" s="16" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D16" s="27" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E16" s="19"/>
     </row>
@@ -1532,23 +2685,23 @@
         <v>21</v>
       </c>
       <c r="C18" s="21" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D18" s="20" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E18" s="19"/>
     </row>
     <row r="19" spans="1:5" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A19" s="32"/>
       <c r="B19" s="22" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C19" s="21" t="s">
         <v>41</v>
       </c>
       <c r="D19" s="21" t="s">
-        <v>63</v>
+        <v>81</v>
       </c>
       <c r="E19" s="25"/>
     </row>
@@ -1563,7 +2716,7 @@
         <v>30</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="E20" s="13" t="s">
         <v>34</v>
@@ -1584,10 +2737,10 @@
         <v>18</v>
       </c>
       <c r="C22" s="28" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D22" s="16" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="E22" s="19"/>
     </row>
@@ -1597,10 +2750,10 @@
         <v>25</v>
       </c>
       <c r="C23" s="21" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D23" s="16" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="E23" s="19"/>
     </row>
@@ -1622,7 +2775,7 @@
         <v>29</v>
       </c>
       <c r="D25" s="30" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E25" s="19"/>
     </row>
@@ -1632,10 +2785,10 @@
         <v>40</v>
       </c>
       <c r="C26" s="21" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D26" s="21" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="E26" s="19"/>
     </row>
@@ -1645,58 +2798,78 @@
         <v>21</v>
       </c>
       <c r="C27" s="21" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D27" s="29" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="E27" s="19"/>
     </row>
     <row r="28" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A28" s="32"/>
       <c r="B28" s="22" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C28" s="21"/>
       <c r="D28" s="21"/>
       <c r="E28" s="25"/>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" ht="87" x14ac:dyDescent="0.35">
       <c r="A29" s="10" t="s">
         <v>5</v>
       </c>
       <c r="B29" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="C29" s="11"/>
-      <c r="D29" s="11"/>
-      <c r="E29" s="13"/>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="C29" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="D29" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="E29" s="33" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="87" x14ac:dyDescent="0.35">
       <c r="A30" s="14"/>
       <c r="B30" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="C30" s="28"/>
-      <c r="D30" s="16"/>
-      <c r="E30" s="18"/>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="C30" s="28" t="s">
+        <v>78</v>
+      </c>
+      <c r="D30" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="E30" s="6" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A31" s="31"/>
       <c r="B31" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="C31" s="28"/>
-      <c r="D31" s="16"/>
+      <c r="C31" s="28" t="s">
+        <v>42</v>
+      </c>
+      <c r="D31" s="34" t="s">
+        <v>85</v>
+      </c>
       <c r="E31" s="19"/>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A32" s="31"/>
       <c r="B32" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="C32" s="21"/>
-      <c r="D32" s="16"/>
+      <c r="C32" s="28" t="s">
+        <v>86</v>
+      </c>
+      <c r="D32" s="34" t="s">
+        <v>87</v>
+      </c>
       <c r="E32" s="19"/>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.35">
@@ -1704,26 +2877,32 @@
       <c r="B33" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="C33" s="16"/>
-      <c r="D33" s="26"/>
       <c r="E33" s="19"/>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A34" s="31"/>
       <c r="B34" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="C34" s="16"/>
-      <c r="D34" s="30"/>
+      <c r="C34" s="28" t="s">
+        <v>42</v>
+      </c>
+      <c r="D34" s="26" t="s">
+        <v>88</v>
+      </c>
       <c r="E34" s="19"/>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" ht="188.5" x14ac:dyDescent="0.35">
       <c r="A35" s="31"/>
       <c r="B35" s="20" t="s">
         <v>40</v>
       </c>
-      <c r="C35" s="21"/>
-      <c r="D35" s="21"/>
+      <c r="C35" s="21" t="s">
+        <v>41</v>
+      </c>
+      <c r="D35" s="21" t="s">
+        <v>90</v>
+      </c>
       <c r="E35" s="19"/>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.35">
@@ -1732,24 +2911,354 @@
         <v>21</v>
       </c>
       <c r="C36" s="21"/>
-      <c r="D36" s="29"/>
+      <c r="D36" s="35" t="s">
+        <v>89</v>
+      </c>
       <c r="E36" s="19"/>
     </row>
     <row r="37" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A37" s="32"/>
       <c r="B37" s="22" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C37" s="21"/>
       <c r="D37" s="21"/>
       <c r="E37" s="25"/>
     </row>
+    <row r="38" spans="1:5" ht="159.5" x14ac:dyDescent="0.35">
+      <c r="A38" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="B38" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="C38" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="D38" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="E38" s="33" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" ht="87" x14ac:dyDescent="0.35">
+      <c r="A39" s="14"/>
+      <c r="B39" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="C39" s="28" t="s">
+        <v>78</v>
+      </c>
+      <c r="D39" s="28" t="s">
+        <v>93</v>
+      </c>
+      <c r="E39" s="6" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" ht="58" x14ac:dyDescent="0.35">
+      <c r="A40" s="31"/>
+      <c r="B40" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="C40" s="28" t="s">
+        <v>42</v>
+      </c>
+      <c r="D40" s="34" t="s">
+        <v>94</v>
+      </c>
+      <c r="E40" s="19"/>
+    </row>
+    <row r="41" spans="1:5" ht="217.5" x14ac:dyDescent="0.35">
+      <c r="A41" s="31"/>
+      <c r="B41" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="C41" s="28" t="s">
+        <v>86</v>
+      </c>
+      <c r="D41" s="34" t="s">
+        <v>95</v>
+      </c>
+      <c r="E41" s="19"/>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A42" s="31"/>
+      <c r="B42" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="E42" s="19"/>
+    </row>
+    <row r="43" spans="1:5" ht="58" x14ac:dyDescent="0.35">
+      <c r="A43" s="31"/>
+      <c r="B43" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="C43" s="28" t="s">
+        <v>42</v>
+      </c>
+      <c r="D43" s="26" t="s">
+        <v>96</v>
+      </c>
+      <c r="E43" s="19"/>
+    </row>
+    <row r="44" spans="1:5" ht="391.5" x14ac:dyDescent="0.35">
+      <c r="A44" s="31"/>
+      <c r="B44" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="C44" s="21" t="s">
+        <v>41</v>
+      </c>
+      <c r="D44" s="21" t="s">
+        <v>97</v>
+      </c>
+      <c r="E44" s="19"/>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A45" s="31"/>
+      <c r="B45" s="20" t="s">
+        <v>21</v>
+      </c>
+      <c r="C45" s="21"/>
+      <c r="D45" s="35" t="s">
+        <v>91</v>
+      </c>
+      <c r="E45" s="19"/>
+    </row>
+    <row r="46" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A46" s="32"/>
+      <c r="B46" s="22" t="s">
+        <v>45</v>
+      </c>
+      <c r="C46" s="21"/>
+      <c r="D46" s="21"/>
+      <c r="E46" s="25"/>
+    </row>
+    <row r="47" spans="1:5" ht="58" x14ac:dyDescent="0.35">
+      <c r="A47" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="B47" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="C47" s="11" t="s">
+        <v>117</v>
+      </c>
+      <c r="D47" s="11" t="s">
+        <v>108</v>
+      </c>
+      <c r="E47" s="33"/>
+    </row>
+    <row r="48" spans="1:5" ht="116" x14ac:dyDescent="0.35">
+      <c r="A48" s="14"/>
+      <c r="B48" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="C48" s="28" t="s">
+        <v>104</v>
+      </c>
+      <c r="D48" s="28" t="s">
+        <v>109</v>
+      </c>
+      <c r="E48" s="6"/>
+    </row>
+    <row r="49" spans="1:5" ht="58" x14ac:dyDescent="0.35">
+      <c r="A49" s="31"/>
+      <c r="B49" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="C49" s="28" t="s">
+        <v>105</v>
+      </c>
+      <c r="D49" s="36" t="s">
+        <v>110</v>
+      </c>
+      <c r="E49" s="19"/>
+    </row>
+    <row r="50" spans="1:5" ht="87" x14ac:dyDescent="0.35">
+      <c r="A50" s="31"/>
+      <c r="B50" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="C50" s="28" t="s">
+        <v>106</v>
+      </c>
+      <c r="D50" s="36" t="s">
+        <v>112</v>
+      </c>
+      <c r="E50" s="19"/>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A51" s="31"/>
+      <c r="B51" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="E51" s="19"/>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A52" s="31"/>
+      <c r="B52" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="C52" s="28" t="s">
+        <v>42</v>
+      </c>
+      <c r="D52" s="26" t="s">
+        <v>107</v>
+      </c>
+      <c r="E52" s="19"/>
+    </row>
+    <row r="53" spans="1:5" ht="87" x14ac:dyDescent="0.35">
+      <c r="A53" s="31"/>
+      <c r="B53" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="C53" s="21" t="s">
+        <v>69</v>
+      </c>
+      <c r="D53" s="21" t="s">
+        <v>111</v>
+      </c>
+      <c r="E53" s="19"/>
+    </row>
+    <row r="54" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A54" s="31"/>
+      <c r="B54" s="20" t="s">
+        <v>21</v>
+      </c>
+      <c r="C54" s="21" t="s">
+        <v>102</v>
+      </c>
+      <c r="D54" s="35" t="s">
+        <v>103</v>
+      </c>
+      <c r="E54" s="19"/>
+    </row>
+    <row r="55" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A55" s="32"/>
+      <c r="B55" s="22" t="s">
+        <v>45</v>
+      </c>
+      <c r="C55" s="21"/>
+      <c r="D55" s="21"/>
+      <c r="E55" s="25"/>
+    </row>
+    <row r="56" spans="1:5" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A56" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="B56" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="C56" s="11" t="s">
+        <v>116</v>
+      </c>
+      <c r="D56" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="E56" s="33"/>
+    </row>
+    <row r="57" spans="1:5" ht="58" x14ac:dyDescent="0.35">
+      <c r="A57" s="14"/>
+      <c r="B57" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="C57" s="28" t="s">
+        <v>119</v>
+      </c>
+      <c r="D57" s="28" t="s">
+        <v>120</v>
+      </c>
+      <c r="E57" s="6"/>
+    </row>
+    <row r="58" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A58" s="31"/>
+      <c r="B58" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="C58" s="28" t="s">
+        <v>42</v>
+      </c>
+      <c r="D58" s="36" t="s">
+        <v>121</v>
+      </c>
+      <c r="E58" s="19"/>
+    </row>
+    <row r="59" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A59" s="31"/>
+      <c r="B59" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="C59" s="28" t="s">
+        <v>42</v>
+      </c>
+      <c r="D59" s="36" t="s">
+        <v>122</v>
+      </c>
+      <c r="E59" s="19"/>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A60" s="31"/>
+      <c r="B60" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="E60" s="19"/>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A61" s="31"/>
+      <c r="B61" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="C61" s="28" t="s">
+        <v>42</v>
+      </c>
+      <c r="D61" s="26" t="s">
+        <v>123</v>
+      </c>
+      <c r="E61" s="19"/>
+    </row>
+    <row r="62" spans="1:5" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A62" s="31"/>
+      <c r="B62" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="C62" s="21"/>
+      <c r="D62" s="21" t="s">
+        <v>124</v>
+      </c>
+      <c r="E62" s="19"/>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A63" s="31"/>
+      <c r="B63" s="20" t="s">
+        <v>21</v>
+      </c>
+      <c r="C63" s="21"/>
+      <c r="D63" s="35">
+        <v>0</v>
+      </c>
+      <c r="E63" s="19"/>
+    </row>
+    <row r="64" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A64" s="32"/>
+      <c r="B64" s="22" t="s">
+        <v>45</v>
+      </c>
+      <c r="C64" s="21"/>
+      <c r="D64" s="21"/>
+      <c r="E64" s="25"/>
+    </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="7">
+    <mergeCell ref="A49:A55"/>
+    <mergeCell ref="A58:A64"/>
     <mergeCell ref="A4:A10"/>
     <mergeCell ref="A13:A19"/>
     <mergeCell ref="A22:A28"/>
     <mergeCell ref="A31:A37"/>
+    <mergeCell ref="A40:A46"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>